<commit_message>
[Progress] accel_fill_sku ถึงหน้ากรอกร SN
</commit_message>
<xml_diff>
--- a/test/tkinter_test/Accel_mode.xlsx
+++ b/test/tkinter_test/Accel_mode.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t xml:space="preserve">orders</t>
   </si>
@@ -29,6 +29,15 @@
   </si>
   <si>
     <t xml:space="preserve">cp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">240329BTB8A373</t>
+  </si>
+  <si>
+    <t xml:space="preserve">evev</t>
+  </si>
+  <si>
+    <t xml:space="preserve">240329C2X8U4H1</t>
   </si>
 </sst>
 </file>
@@ -49,16 +58,19 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+      <charset val="222"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+      <charset val="222"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+      <charset val="222"/>
     </font>
   </fonts>
   <fills count="2">
@@ -130,7 +142,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22.39"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="31.57"/>
@@ -147,7 +159,18 @@
         <v>2</v>
       </c>
     </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>4</v>
+      </c>
+    </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="s">
+        <v>5</v>
+      </c>
       <c r="B3" s="1"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -161,8 +184,8 @@
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,ปกติ"&amp;12&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,ปกติ"&amp;12Page &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[progress] accelmode autoadd item by sn
</commit_message>
<xml_diff>
--- a/test/tkinter_test/Accel_mode.xlsx
+++ b/test/tkinter_test/Accel_mode.xlsx
@@ -8,7 +8,7 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId2"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t xml:space="preserve">orders</t>
   </si>
@@ -31,16 +31,25 @@
     <t xml:space="preserve">cp</t>
   </si>
   <si>
-    <t xml:space="preserve">240329BTB8A373</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E80714F3H493786 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">240329C2X8U4H1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E80714H3H189597 </t>
+    <t xml:space="preserve">240404S3WV2T9J</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BB3H133801428 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">CP2404010041 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">240404S6D047VD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BB3H133801408 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">240404SAFEC473</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BB3H133803171 </t>
   </si>
 </sst>
 </file>
@@ -61,16 +70,19 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+      <charset val="222"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+      <charset val="222"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+      <charset val="222"/>
     </font>
   </fonts>
   <fills count="2">
@@ -144,122 +156,17 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
-  <a:themeElements>
-    <a:clrScheme name="LibreOffice">
-      <a:dk1>
-        <a:srgbClr val="000000"/>
-      </a:dk1>
-      <a:lt1>
-        <a:srgbClr val="ffffff"/>
-      </a:lt1>
-      <a:dk2>
-        <a:srgbClr val="000000"/>
-      </a:dk2>
-      <a:lt2>
-        <a:srgbClr val="ffffff"/>
-      </a:lt2>
-      <a:accent1>
-        <a:srgbClr val="18a303"/>
-      </a:accent1>
-      <a:accent2>
-        <a:srgbClr val="0369a3"/>
-      </a:accent2>
-      <a:accent3>
-        <a:srgbClr val="a33e03"/>
-      </a:accent3>
-      <a:accent4>
-        <a:srgbClr val="8e03a3"/>
-      </a:accent4>
-      <a:accent5>
-        <a:srgbClr val="c99c00"/>
-      </a:accent5>
-      <a:accent6>
-        <a:srgbClr val="c9211e"/>
-      </a:accent6>
-      <a:hlink>
-        <a:srgbClr val="0000ee"/>
-      </a:hlink>
-      <a:folHlink>
-        <a:srgbClr val="551a8b"/>
-      </a:folHlink>
-    </a:clrScheme>
-    <a:fontScheme name="Office">
-      <a:majorFont>
-        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
-        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
-        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-      </a:minorFont>
-    </a:fontScheme>
-    <a:fmtScheme>
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
-          <a:prstDash val="solid"/>
-          <a:miter/>
-        </a:ln>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
-          <a:prstDash val="solid"/>
-          <a:miter/>
-        </a:ln>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
-          <a:prstDash val="solid"/>
-          <a:miter/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:bgFillStyleLst>
-    </a:fmtScheme>
-  </a:themeElements>
-</a:theme>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22.39"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="31.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="15.69"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -280,17 +187,25 @@
       <c r="B2" s="2" t="s">
         <v>4</v>
       </c>
+      <c r="C2" s="2" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="3"/>
+      <c r="A4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="3"/>

</xml_diff>

<commit_message>
update remove unneceesary \s in item name
</commit_message>
<xml_diff>
--- a/test/tkinter_test/Accel_mode.xlsx
+++ b/test/tkinter_test/Accel_mode.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t xml:space="preserve">orders</t>
   </si>
@@ -29,40 +29,19 @@
     <t xml:space="preserve">cp</t>
   </si>
   <si>
-    <t xml:space="preserve">240606A59K7J5Q</t>
-  </si>
-  <si>
-    <t xml:space="preserve">240606A72NFNHQ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">240606A9TY9F89</t>
-  </si>
-  <si>
-    <t xml:space="preserve">240606A6N3HPPG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">240606A1XDSANK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">240606A8VR7GR6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">240606A59WQTSF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">240606A60ATX21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">240606A96HXY8S</t>
-  </si>
-  <si>
-    <t xml:space="preserve">240606A5PM05UK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2406058D69V3MA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2406069N5BMMKC</t>
+    <t xml:space="preserve">240606A002Q4CT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">240606B3F76NV4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">240606B4A1JR78</t>
+  </si>
+  <si>
+    <t xml:space="preserve">240606B5E95VF6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">240606AHBP3HQ4</t>
   </si>
 </sst>
 </file>
@@ -78,6 +57,7 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -137,7 +117,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -148,6 +128,14 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -167,12 +155,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
-  <sheetFormatPr defaultColWidth="8.70703125" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:H34"/>
+  <sheetFormatPr defaultColWidth="8.73046875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="31.58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="4" style="1" width="29.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="2" style="1" width="29.03"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -183,107 +170,127 @@
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="0"/>
-      <c r="C2" s="0"/>
-      <c r="E2" s="0"/>
-      <c r="F2" s="0"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="0"/>
-      <c r="E3" s="0"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="0"/>
-      <c r="C4" s="0"/>
-      <c r="D4" s="0"/>
-      <c r="E4" s="0"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="0"/>
-      <c r="C5" s="0"/>
-      <c r="D5" s="0"/>
-      <c r="E5" s="0"/>
-      <c r="F5" s="0"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="0"/>
-      <c r="C6" s="0"/>
-      <c r="D6" s="0"/>
-      <c r="E6" s="0"/>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7" s="0"/>
-      <c r="C7" s="0"/>
-      <c r="D7" s="0"/>
-      <c r="E7" s="0"/>
+      <c r="A7" s="3"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="s">
-        <v>8</v>
-      </c>
       <c r="B8" s="0"/>
       <c r="C8" s="0"/>
-      <c r="D8" s="0"/>
-      <c r="E8" s="0"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="s">
-        <v>9</v>
-      </c>
       <c r="B9" s="0"/>
       <c r="C9" s="0"/>
       <c r="D9" s="0"/>
       <c r="E9" s="0"/>
+      <c r="F9" s="0"/>
+      <c r="G9" s="0"/>
+      <c r="H9" s="0"/>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="1" t="s">
-        <v>10</v>
-      </c>
+      <c r="A10" s="3"/>
       <c r="B10" s="0"/>
       <c r="C10" s="0"/>
       <c r="D10" s="0"/>
       <c r="E10" s="0"/>
+      <c r="F10" s="0"/>
+      <c r="G10" s="0"/>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
-        <v>11</v>
-      </c>
+      <c r="A11" s="3"/>
+      <c r="B11" s="0"/>
+      <c r="C11" s="0"/>
+      <c r="D11" s="0"/>
       <c r="E11" s="0"/>
+      <c r="F11" s="0"/>
+      <c r="G11" s="0"/>
+      <c r="H11" s="0"/>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
-        <v>12</v>
-      </c>
+      <c r="A12" s="0"/>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
       <c r="D12" s="0"/>
       <c r="E12" s="0"/>
+      <c r="F12" s="0"/>
+      <c r="G12" s="3"/>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
-        <v>13</v>
-      </c>
+      <c r="A13" s="0"/>
+      <c r="B13" s="0"/>
+      <c r="C13" s="0"/>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0"/>
@@ -299,9 +306,61 @@
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0"/>
+      <c r="B18" s="0"/>
+      <c r="C18" s="0"/>
+      <c r="D18" s="0"/>
+      <c r="E18" s="0"/>
+      <c r="F18" s="0"/>
+      <c r="G18" s="0"/>
+      <c r="H18" s="0"/>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0"/>
+    </row>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="0"/>
+    </row>
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="0"/>
+    </row>
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="0"/>
+    </row>
+    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="0"/>
+    </row>
+    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="0"/>
+    </row>
+    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="0"/>
+    </row>
+    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="0"/>
+    </row>
+    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="0"/>
+    </row>
+    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="0"/>
+    </row>
+    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="0"/>
+    </row>
+    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="0"/>
+    </row>
+    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="0"/>
+    </row>
+    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="0"/>
+    </row>
+    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="0"/>
+    </row>
+    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="0"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -320,7 +379,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="0.7875" bottom="0.7875" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
wip: flow design for auto fillable product
-คล้ายๆ accel mode
</commit_message>
<xml_diff>
--- a/test/tkinter_test/Accel_mode.xlsx
+++ b/test/tkinter_test/Accel_mode.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -504,6 +504,90 @@
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr"/>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+      <c r="B18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr"/>
+      <c r="B19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr"/>
+      <c r="B20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr"/>
+      <c r="B21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr"/>
+      <c r="B22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr"/>
+      <c r="B23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr"/>
+      <c r="B24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr"/>
+      <c r="B25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr"/>
+      <c r="B26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr"/>
+      <c r="B27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr"/>
+      <c r="B28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr"/>
+      <c r="B29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr"/>
+      <c r="B30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr"/>
+      <c r="B31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr"/>
+      <c r="B32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr"/>
+      <c r="B33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr"/>
+      <c r="B34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr"/>
+      <c r="B35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr"/>
+      <c r="B36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr"/>
+      <c r="B37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr"/>
+      <c r="B38" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>